<commit_message>
generacion especifica de graficos burbuja
</commit_message>
<xml_diff>
--- a/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
+++ b/datasets/datasets_aumentados/logs/pcsmote/por_muestras/log_pcsmote_x_muestra_ecoli.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos_D\etapa-analisis_pcsmote\datasets\datasets_aumentados\logs\pcsmote\por_muestras\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FamiliaNatelloMedina\Desktop\codigo\datasets\datasets_aumentados\logs\pcsmote\por_muestras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BF896A-9055-43B8-8E40-AEBB20B88170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -157,7 +156,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -237,9 +236,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -277,9 +276,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -314,7 +313,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -349,7 +348,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -522,7 +521,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -31001,7 +31000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="430" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
         <v>28</v>
       </c>
@@ -31155,7 +31154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="432" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
         <v>28</v>
       </c>
@@ -31232,7 +31231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="433" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
         <v>28</v>
       </c>
@@ -31463,7 +31462,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="436" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
         <v>28</v>
       </c>
@@ -31617,7 +31616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="438" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
         <v>28</v>
       </c>
@@ -31694,7 +31693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="439" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
         <v>28</v>
       </c>
@@ -31848,7 +31847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="441" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
         <v>28</v>
       </c>
@@ -32002,7 +32001,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="443" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
         <v>28</v>
       </c>
@@ -32156,7 +32155,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="445" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>28</v>
       </c>
@@ -32233,7 +32232,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="446" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
         <v>28</v>
       </c>
@@ -32310,7 +32309,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="447" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
         <v>28</v>
       </c>
@@ -32464,7 +32463,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="449" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
         <v>28</v>
       </c>
@@ -32541,7 +32540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="450" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
         <v>28</v>
       </c>
@@ -32618,7 +32617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="451" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
         <v>28</v>
       </c>
@@ -32695,7 +32694,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="452" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
         <v>28</v>
       </c>
@@ -32772,7 +32771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="453" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
         <v>28</v>
       </c>
@@ -33157,7 +33156,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="458" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
         <v>28</v>
       </c>
@@ -33619,7 +33618,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="464" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
         <v>28</v>
       </c>
@@ -33773,7 +33772,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="466" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
         <v>28</v>
       </c>
@@ -33850,7 +33849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="467" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
         <v>28</v>
       </c>
@@ -33927,7 +33926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="468" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
         <v>28</v>
       </c>
@@ -34081,7 +34080,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="470" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
         <v>28</v>
       </c>
@@ -34158,7 +34157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="471" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
         <v>28</v>
       </c>
@@ -34235,7 +34234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="472" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
         <v>28</v>
       </c>
@@ -34312,7 +34311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="473" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
         <v>28</v>
       </c>
@@ -34389,7 +34388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="474" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
         <v>28</v>
       </c>
@@ -34466,7 +34465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="475" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
         <v>28</v>
       </c>
@@ -34543,7 +34542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="476" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
         <v>28</v>
       </c>
@@ -34620,7 +34619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="477" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
         <v>28</v>
       </c>
@@ -34697,7 +34696,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="478" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
         <v>28</v>
       </c>
@@ -34774,7 +34773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="479" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
         <v>28</v>
       </c>
@@ -34851,7 +34850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="480" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
         <v>28</v>
       </c>
@@ -35082,7 +35081,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="483" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
         <v>28</v>
       </c>
@@ -35313,7 +35312,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="486" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
         <v>28</v>
       </c>
@@ -35390,7 +35389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="487" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
         <v>28</v>
       </c>
@@ -35467,7 +35466,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="488" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
         <v>28</v>
       </c>
@@ -35544,7 +35543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="489" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
         <v>28</v>
       </c>
@@ -35698,7 +35697,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="491" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
         <v>28</v>
       </c>
@@ -35775,7 +35774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="492" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
         <v>28</v>
       </c>
@@ -35852,7 +35851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="493" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
         <v>28</v>
       </c>
@@ -35929,7 +35928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="494" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
         <v>28</v>
       </c>
@@ -36083,7 +36082,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="496" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
         <v>28</v>
       </c>
@@ -36160,7 +36159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="497" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
         <v>28</v>
       </c>
@@ -36237,7 +36236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="498" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
         <v>28</v>
       </c>
@@ -36314,7 +36313,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="499" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
         <v>28</v>
       </c>
@@ -36391,7 +36390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="500" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
         <v>28</v>
       </c>
@@ -36468,7 +36467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="501" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
         <v>28</v>
       </c>
@@ -36853,7 +36852,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="506" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="506" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
         <v>28</v>
       </c>
@@ -36930,7 +36929,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="507" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="507" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
         <v>28</v>
       </c>
@@ -37392,7 +37391,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="513" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="513" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A513" t="s">
         <v>28</v>
       </c>
@@ -37546,7 +37545,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="515" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="515" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A515" t="s">
         <v>28</v>
       </c>
@@ -37623,7 +37622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="516" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="516" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A516" t="s">
         <v>28</v>
       </c>
@@ -37700,7 +37699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="517" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="517" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A517" t="s">
         <v>28</v>
       </c>
@@ -37777,7 +37776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="518" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="518" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A518" t="s">
         <v>28</v>
       </c>
@@ -38162,7 +38161,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="523" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="523" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A523" t="s">
         <v>28</v>
       </c>
@@ -38239,7 +38238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="524" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="524" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A524" t="s">
         <v>28</v>
       </c>
@@ -38316,7 +38315,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="525" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="525" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
         <v>28</v>
       </c>
@@ -38393,7 +38392,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="526" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="526" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
         <v>28</v>
       </c>
@@ -38470,7 +38469,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="527" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="527" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
         <v>28</v>
       </c>
@@ -38547,7 +38546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="528" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="528" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
         <v>28</v>
       </c>
@@ -38624,7 +38623,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="529" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="529" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
         <v>28</v>
       </c>
@@ -38701,7 +38700,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="530" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="530" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
         <v>28</v>
       </c>
@@ -38778,7 +38777,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="531" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="531" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
         <v>28</v>
       </c>
@@ -38855,7 +38854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="532" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="532" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
         <v>28</v>
       </c>
@@ -38932,7 +38931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="533" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="533" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
         <v>28</v>
       </c>
@@ -39009,7 +39008,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="534" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="534" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
         <v>28</v>
       </c>
@@ -39163,7 +39162,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="536" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="536" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
         <v>28</v>
       </c>
@@ -39240,7 +39239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="537" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="537" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
         <v>28</v>
       </c>
@@ -39471,7 +39470,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="540" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="540" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
         <v>28</v>
       </c>
@@ -39548,7 +39547,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="541" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="541" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
         <v>28</v>
       </c>
@@ -39702,7 +39701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="543" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="543" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
         <v>28</v>
       </c>
@@ -39779,7 +39778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="544" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="544" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A544" t="s">
         <v>28</v>
       </c>
@@ -40010,7 +40009,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="547" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="547" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A547" t="s">
         <v>28</v>
       </c>
@@ -40087,7 +40086,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="548" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="548" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A548" t="s">
         <v>28</v>
       </c>
@@ -40164,7 +40163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="549" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="549" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A549" t="s">
         <v>28</v>
       </c>
@@ -40241,7 +40240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="550" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="550" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A550" t="s">
         <v>28</v>
       </c>
@@ -40318,7 +40317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="551" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="551" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
         <v>28</v>
       </c>
@@ -40395,7 +40394,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="552" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="552" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A552" t="s">
         <v>28</v>
       </c>
@@ -40472,7 +40471,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="553" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="553" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A553" t="s">
         <v>28</v>
       </c>
@@ -40626,7 +40625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="555" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="555" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A555" t="s">
         <v>28</v>
       </c>
@@ -40703,7 +40702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="556" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="556" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A556" t="s">
         <v>28</v>
       </c>
@@ -40857,7 +40856,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="558" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="558" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A558" t="s">
         <v>28</v>
       </c>
@@ -40934,7 +40933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="559" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="559" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A559" t="s">
         <v>28</v>
       </c>
@@ -41319,7 +41318,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="564" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="564" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A564" t="s">
         <v>28</v>
       </c>
@@ -41473,7 +41472,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="566" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="566" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
         <v>28</v>
       </c>
@@ -41627,7 +41626,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="568" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="568" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A568" t="s">
         <v>28</v>
       </c>
@@ -41704,7 +41703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="569" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="569" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A569" t="s">
         <v>28</v>
       </c>
@@ -41781,7 +41780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="570" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="570" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A570" t="s">
         <v>28</v>
       </c>
@@ -41858,7 +41857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="571" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A571" t="s">
         <v>28</v>
       </c>
@@ -42089,7 +42088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="574" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A574" t="s">
         <v>28</v>
       </c>
@@ -42166,7 +42165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="575" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
+    <row r="575" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A575" t="s">
         <v>28</v>
       </c>
@@ -42320,7 +42319,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="577" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="577" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A577" t="s">
         <v>29</v>
       </c>
@@ -42551,7 +42550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="580" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="580" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A580" t="s">
         <v>29</v>
       </c>
@@ -42628,7 +42627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="581" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="581" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A581" t="s">
         <v>29</v>
       </c>
@@ -42782,7 +42781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="583" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="583" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A583" t="s">
         <v>29</v>
       </c>
@@ -43013,7 +43012,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="586" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="586" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A586" t="s">
         <v>29</v>
       </c>
@@ -43167,7 +43166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="588" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="588" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A588" t="s">
         <v>29</v>
       </c>
@@ -43321,7 +43320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="590" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="590" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A590" t="s">
         <v>29</v>
       </c>
@@ -43629,7 +43628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="594" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="594" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A594" t="s">
         <v>29</v>
       </c>
@@ -44091,7 +44090,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="600" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="600" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A600" t="s">
         <v>29</v>
       </c>
@@ -44168,7 +44167,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="601" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="601" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A601" t="s">
         <v>29</v>
       </c>
@@ -44245,7 +44244,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="602" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="602" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A602" t="s">
         <v>29</v>
       </c>
@@ -44322,7 +44321,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="603" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="603" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A603" t="s">
         <v>29</v>
       </c>
@@ -44476,7 +44475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="605" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="605" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A605" t="s">
         <v>29</v>
       </c>
@@ -44553,7 +44552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="606" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="606" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A606" t="s">
         <v>29</v>
       </c>
@@ -44630,7 +44629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="607" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="607" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A607" t="s">
         <v>29</v>
       </c>
@@ -44707,7 +44706,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="608" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="608" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A608" t="s">
         <v>29</v>
       </c>
@@ -44784,7 +44783,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="609" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="609" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A609" t="s">
         <v>29</v>
       </c>
@@ -44938,7 +44937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="611" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="611" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A611" t="s">
         <v>29</v>
       </c>
@@ -45246,7 +45245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="615" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="615" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A615" t="s">
         <v>29</v>
       </c>
@@ -46170,7 +46169,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="627" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="627" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A627" t="s">
         <v>29</v>
       </c>
@@ -46247,7 +46246,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="628" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="628" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A628" t="s">
         <v>29</v>
       </c>
@@ -46478,7 +46477,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="631" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="631" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A631" t="s">
         <v>29</v>
       </c>
@@ -46786,7 +46785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="635" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="635" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A635" t="s">
         <v>29</v>
       </c>
@@ -47094,7 +47093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="639" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="639" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A639" t="s">
         <v>29</v>
       </c>
@@ -47633,7 +47632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="646" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="646" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A646" t="s">
         <v>29</v>
       </c>
@@ -47710,7 +47709,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="647" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="647" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A647" t="s">
         <v>29</v>
       </c>
@@ -47787,7 +47786,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="648" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="648" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A648" t="s">
         <v>29</v>
       </c>
@@ -47864,7 +47863,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="649" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="649" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A649" t="s">
         <v>29</v>
       </c>
@@ -48095,7 +48094,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="652" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="652" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A652" t="s">
         <v>29</v>
       </c>
@@ -48172,7 +48171,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="653" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="653" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A653" t="s">
         <v>29</v>
       </c>
@@ -48249,7 +48248,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="654" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="654" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A654" t="s">
         <v>29</v>
       </c>
@@ -48403,7 +48402,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="656" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="656" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A656" t="s">
         <v>29</v>
       </c>
@@ -48557,7 +48556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="658" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="658" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A658" t="s">
         <v>29</v>
       </c>
@@ -49096,7 +49095,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="665" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="665" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A665" t="s">
         <v>29</v>
       </c>
@@ -49173,7 +49172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="666" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="666" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A666" t="s">
         <v>29</v>
       </c>
@@ -50097,7 +50096,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="678" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="678" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A678" t="s">
         <v>29</v>
       </c>
@@ -50328,7 +50327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="681" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="681" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A681" t="s">
         <v>29</v>
       </c>
@@ -50405,7 +50404,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="682" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="682" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A682" t="s">
         <v>29</v>
       </c>
@@ -50636,7 +50635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="685" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="685" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A685" t="s">
         <v>29</v>
       </c>
@@ -50867,7 +50866,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="688" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="688" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A688" t="s">
         <v>29</v>
       </c>
@@ -50944,7 +50943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="689" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="689" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A689" t="s">
         <v>29</v>
       </c>
@@ -51560,7 +51559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="697" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="697" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A697" t="s">
         <v>29</v>
       </c>
@@ -51791,7 +51790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="700" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="700" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A700" t="s">
         <v>29</v>
       </c>
@@ -52022,7 +52021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="703" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="703" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A703" t="s">
         <v>29</v>
       </c>
@@ -52099,7 +52098,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="704" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="704" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A704" t="s">
         <v>29</v>
       </c>
@@ -52176,7 +52175,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="705" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="705" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A705" t="s">
         <v>29</v>
       </c>
@@ -52253,7 +52252,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="706" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="706" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A706" t="s">
         <v>29</v>
       </c>
@@ -52407,7 +52406,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="708" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="708" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A708" t="s">
         <v>29</v>
       </c>
@@ -52561,7 +52560,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="710" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="710" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A710" t="s">
         <v>29</v>
       </c>
@@ -52869,7 +52868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="714" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="714" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A714" t="s">
         <v>29</v>
       </c>
@@ -52946,7 +52945,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="715" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="715" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A715" t="s">
         <v>29</v>
       </c>
@@ -53178,13 +53177,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y717" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="3">
+  <autoFilter ref="A1:Y717">
+    <filterColumn colId="0">
       <filters>
-        <filter val="VERDADERO"/>
+        <filter val="PRD70_PR40_CPent_UD060_UR045_PE60_I0"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A431:Y573">
+    <sortState ref="A431:Y573">
       <sortCondition descending="1" ref="W1:W717"/>
     </sortState>
   </autoFilter>

</xml_diff>